<commit_message>
rm old mapping 7d14d3abcd5beae642da20b2dd28be157ec4e197
</commit_message>
<xml_diff>
--- a/nr-add-mapping/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/nr-add-mapping/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Internal Id Systems</t>
+    <t>AS CodeSystem Internal Identifier Systems</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-05T10:02:39+00:00</t>
+    <t>2024-03-19T08:59:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Systèmes des identifiants locaux</t>
+    <t>CodeSystem contenant les identifiants locaux</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>